<commit_message>
Add Planner v2 repository diagnostics with bounded recovery and signed replay
</commit_message>
<xml_diff>
--- a/project/StellaDev WBSO 2026 - Hours registration -  (ENG).xlsx
+++ b/project/StellaDev WBSO 2026 - Hours registration -  (ENG).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10810"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10920"/>
   <workbookPr checkCompatibility="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/filippomargiotta/Documents/Personal/AosRepo/project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AE9F975-D970-DC42-98A0-07B9327A252A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02A111C5-828C-2943-AA2E-04B4AFE8C2A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="33320" windowHeight="17620" tabRatio="666" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="580" windowWidth="29920" windowHeight="17620" tabRatio="666" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="2" r:id="rId1"/>
@@ -2099,7 +2099,7 @@
       </c>
       <c r="K12" s="70">
         <f>September!AG14</f>
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="L12" s="70">
         <f>October!AH14</f>
@@ -2115,7 +2115,7 @@
       </c>
       <c r="O12" s="69">
         <f>SUM(C12:N12)</f>
-        <v>772</v>
+        <v>862</v>
       </c>
     </row>
     <row r="13" spans="1:34" ht="15" customHeight="1">
@@ -3084,7 +3084,7 @@
       </c>
       <c r="K29" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="L29" s="5">
         <f t="shared" si="1"/>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="O29" s="6">
         <f t="shared" si="1"/>
-        <v>772</v>
+        <v>862</v>
       </c>
     </row>
     <row r="31" spans="2:15" ht="15" customHeight="1">
@@ -3405,39 +3405,85 @@
         <f>January!B14</f>
         <v>AI-Driven Agentic Orchestration Software (AOC-WebAPI)</v>
       </c>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
+      <c r="C14" s="17">
+        <v>4</v>
+      </c>
+      <c r="D14" s="17">
+        <v>3</v>
+      </c>
       <c r="E14" s="17"/>
-      <c r="F14" s="17"/>
-      <c r="G14" s="18"/>
+      <c r="F14" s="17">
+        <v>4</v>
+      </c>
+      <c r="G14" s="18">
+        <v>5</v>
+      </c>
       <c r="H14" s="16"/>
-      <c r="I14" s="17"/>
-      <c r="J14" s="17"/>
+      <c r="I14" s="17">
+        <v>5</v>
+      </c>
+      <c r="J14" s="17">
+        <v>6</v>
+      </c>
       <c r="K14" s="17"/>
-      <c r="L14" s="17"/>
+      <c r="L14" s="17">
+        <v>2</v>
+      </c>
       <c r="M14" s="17"/>
-      <c r="N14" s="18"/>
-      <c r="O14" s="16"/>
-      <c r="P14" s="17"/>
-      <c r="Q14" s="17"/>
+      <c r="N14" s="18">
+        <v>6</v>
+      </c>
+      <c r="O14" s="16">
+        <v>4</v>
+      </c>
+      <c r="P14" s="17">
+        <v>4</v>
+      </c>
+      <c r="Q14" s="17">
+        <v>4</v>
+      </c>
       <c r="R14" s="17"/>
-      <c r="S14" s="17"/>
-      <c r="T14" s="17"/>
-      <c r="U14" s="18"/>
+      <c r="S14" s="17">
+        <v>3</v>
+      </c>
+      <c r="T14" s="17">
+        <v>5</v>
+      </c>
+      <c r="U14" s="18">
+        <v>2</v>
+      </c>
       <c r="V14" s="16"/>
-      <c r="W14" s="17"/>
-      <c r="X14" s="17"/>
-      <c r="Y14" s="17"/>
+      <c r="W14" s="17">
+        <v>4</v>
+      </c>
+      <c r="X14" s="17">
+        <v>4</v>
+      </c>
+      <c r="Y14" s="17">
+        <v>2</v>
+      </c>
       <c r="Z14" s="17"/>
-      <c r="AA14" s="17"/>
-      <c r="AB14" s="18"/>
-      <c r="AC14" s="16"/>
-      <c r="AD14" s="17"/>
-      <c r="AE14" s="17"/>
-      <c r="AF14" s="20"/>
+      <c r="AA14" s="17">
+        <v>5</v>
+      </c>
+      <c r="AB14" s="18">
+        <v>4</v>
+      </c>
+      <c r="AC14" s="16">
+        <v>4</v>
+      </c>
+      <c r="AD14" s="17">
+        <v>2</v>
+      </c>
+      <c r="AE14" s="17">
+        <v>4</v>
+      </c>
+      <c r="AF14" s="20">
+        <v>4</v>
+      </c>
       <c r="AG14" s="43">
         <f t="shared" ref="AG14:AG30" si="0">SUM(C14:AF14)</f>
-        <v>0</v>
+        <v>90</v>
       </c>
     </row>
     <row r="15" spans="1:33" ht="15" customHeight="1">
@@ -17350,15 +17396,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="0e61e294-5db2-4ad2-9356-7488524978e7">
@@ -17367,6 +17404,15 @@
     <TaxCatchAll xmlns="9160ec49-0786-419e-aae3-9c9cb8f5a974" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -17389,14 +17435,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D23919C5-C77D-4D6C-8993-5ED5B021C1A8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1149BA22-2185-4279-8D4D-20B81C2A7999}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -17409,6 +17447,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D23919C5-C77D-4D6C-8993-5ED5B021C1A8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{0eea11ca-d417-4147-80ed-01a58412c458}" enabled="1" method="Standard" siteId="{bc9dc15c-61bc-4f03-b60b-e5b6d8922839}" contentBits="2" removed="0"/>

</xml_diff>

<commit_message>
Add RDI-08/11/12: ambiguity, network denial, snapshot-free replay
</commit_message>
<xml_diff>
--- a/project/StellaDev WBSO 2026 - Hours registration -  (ENG).xlsx
+++ b/project/StellaDev WBSO 2026 - Hours registration -  (ENG).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10920"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10927"/>
   <workbookPr checkCompatibility="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/filippomargiotta/Documents/Personal/AosRepo/project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02A111C5-828C-2943-AA2E-04B4AFE8C2A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{502BAF2D-5385-8044-BF3B-91B4208FB978}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="580" windowWidth="29920" windowHeight="17620" tabRatio="666" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29920" windowHeight="17620" tabRatio="666" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="2" r:id="rId1"/>
@@ -2103,7 +2103,7 @@
       </c>
       <c r="L12" s="70">
         <f>October!AH14</f>
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="M12" s="70">
         <f>November!AG14</f>
@@ -2115,7 +2115,7 @@
       </c>
       <c r="O12" s="69">
         <f>SUM(C12:N12)</f>
-        <v>862</v>
+        <v>908</v>
       </c>
     </row>
     <row r="13" spans="1:34" ht="15" customHeight="1">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="L29" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="M29" s="5">
         <f t="shared" si="1"/>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="O29" s="6">
         <f t="shared" si="1"/>
-        <v>862</v>
+        <v>908</v>
       </c>
     </row>
     <row r="31" spans="2:15" ht="15" customHeight="1">
@@ -4577,20 +4577,42 @@
         <f>January!B14</f>
         <v>AI-Driven Agentic Orchestration Software (AOC-WebAPI)</v>
       </c>
-      <c r="C14" s="41"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="18"/>
+      <c r="C14" s="41">
+        <v>4</v>
+      </c>
+      <c r="D14" s="17">
+        <v>6</v>
+      </c>
+      <c r="E14" s="18">
+        <v>2</v>
+      </c>
       <c r="F14" s="16"/>
-      <c r="G14" s="17"/>
-      <c r="H14" s="17"/>
-      <c r="I14" s="17"/>
-      <c r="J14" s="17"/>
-      <c r="K14" s="17"/>
+      <c r="G14" s="17">
+        <v>4</v>
+      </c>
+      <c r="H14" s="17">
+        <v>4</v>
+      </c>
+      <c r="I14" s="17">
+        <v>6</v>
+      </c>
+      <c r="J14" s="17">
+        <v>4</v>
+      </c>
+      <c r="K14" s="17">
+        <v>4</v>
+      </c>
       <c r="L14" s="18"/>
-      <c r="M14" s="16"/>
+      <c r="M14" s="16">
+        <v>2</v>
+      </c>
       <c r="N14" s="17"/>
-      <c r="O14" s="17"/>
-      <c r="P14" s="17"/>
+      <c r="O14" s="17">
+        <v>6</v>
+      </c>
+      <c r="P14" s="17">
+        <v>4</v>
+      </c>
       <c r="Q14" s="17"/>
       <c r="R14" s="17"/>
       <c r="S14" s="18"/>
@@ -4610,7 +4632,7 @@
       <c r="AG14" s="54"/>
       <c r="AH14" s="43">
         <f>SUM(C14:AG14)</f>
-        <v>0</v>
+        <v>46</v>
       </c>
     </row>
     <row r="15" spans="1:34" ht="15" customHeight="1">
@@ -17161,6 +17183,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0e61e294-5db2-4ad2-9356-7488524978e7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9160ec49-0786-419e-aae3-9c9cb8f5a974" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C289070B8F9CFE47959C16D84F6C625E" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="fe8aa3d2fe1a9c7effcd8e73d8f32c18">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0e61e294-5db2-4ad2-9356-7488524978e7" xmlns:ns3="9160ec49-0786-419e-aae3-9c9cb8f5a974" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d0f39d0209994a88c6a94a692ea058f4" ns2:_="" ns3:_="">
     <xsd:import namespace="0e61e294-5db2-4ad2-9356-7488524978e7"/>
@@ -17395,27 +17437,28 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0e61e294-5db2-4ad2-9356-7488524978e7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9160ec49-0786-419e-aae3-9c9cb8f5a974" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D23919C5-C77D-4D6C-8993-5ED5B021C1A8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1149BA22-2185-4279-8D4D-20B81C2A7999}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="a022c38d-a398-45a6-8336-4b22e89f761d"/>
+    <ds:schemaRef ds:uri="52db9a4d-0878-46fa-948e-68042efe192b"/>
+    <ds:schemaRef ds:uri="0e61e294-5db2-4ad2-9356-7488524978e7"/>
+    <ds:schemaRef ds:uri="9160ec49-0786-419e-aae3-9c9cb8f5a974"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2824570A-9196-4B56-8A33-38A1E7BF27D2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -17434,27 +17477,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1149BA22-2185-4279-8D4D-20B81C2A7999}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="a022c38d-a398-45a6-8336-4b22e89f761d"/>
-    <ds:schemaRef ds:uri="52db9a4d-0878-46fa-948e-68042efe192b"/>
-    <ds:schemaRef ds:uri="0e61e294-5db2-4ad2-9356-7488524978e7"/>
-    <ds:schemaRef ds:uri="9160ec49-0786-419e-aae3-9c9cb8f5a974"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D23919C5-C77D-4D6C-8993-5ED5B021C1A8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{0eea11ca-d417-4147-80ed-01a58412c458}" enabled="1" method="Standard" siteId="{bc9dc15c-61bc-4f03-b60b-e5b6d8922839}" contentBits="2" removed="0"/>

</xml_diff>

<commit_message>
Add fixture v2 (RDI-03/04/05), semantic scoring, and per-stage regression gate
</commit_message>
<xml_diff>
--- a/project/StellaDev WBSO 2026 - Hours registration -  (ENG).xlsx
+++ b/project/StellaDev WBSO 2026 - Hours registration -  (ENG).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/filippomargiotta/Documents/Personal/AosRepo/project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{502BAF2D-5385-8044-BF3B-91B4208FB978}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{321B8E83-E169-C14C-A022-8036F34741DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29920" windowHeight="17620" tabRatio="666" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="32200" windowHeight="19920" tabRatio="666" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="2" r:id="rId1"/>
@@ -2103,7 +2103,7 @@
       </c>
       <c r="L12" s="70">
         <f>October!AH14</f>
-        <v>46</v>
+        <v>73</v>
       </c>
       <c r="M12" s="70">
         <f>November!AG14</f>
@@ -2115,7 +2115,7 @@
       </c>
       <c r="O12" s="69">
         <f>SUM(C12:N12)</f>
-        <v>908</v>
+        <v>935</v>
       </c>
     </row>
     <row r="13" spans="1:34" ht="15" customHeight="1">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="L29" s="5">
         <f t="shared" si="1"/>
-        <v>46</v>
+        <v>73</v>
       </c>
       <c r="M29" s="5">
         <f t="shared" si="1"/>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="O29" s="6">
         <f t="shared" si="1"/>
-        <v>908</v>
+        <v>935</v>
       </c>
     </row>
     <row r="31" spans="2:15" ht="15" customHeight="1">
@@ -4614,14 +4614,28 @@
         <v>4</v>
       </c>
       <c r="Q14" s="17"/>
-      <c r="R14" s="17"/>
-      <c r="S14" s="18"/>
+      <c r="R14" s="17">
+        <v>4</v>
+      </c>
+      <c r="S14" s="18">
+        <v>3</v>
+      </c>
       <c r="T14" s="16"/>
-      <c r="U14" s="17"/>
-      <c r="V14" s="17"/>
-      <c r="W14" s="17"/>
-      <c r="X14" s="17"/>
-      <c r="Y14" s="17"/>
+      <c r="U14" s="17">
+        <v>4</v>
+      </c>
+      <c r="V14" s="17">
+        <v>2</v>
+      </c>
+      <c r="W14" s="17">
+        <v>4</v>
+      </c>
+      <c r="X14" s="17">
+        <v>4</v>
+      </c>
+      <c r="Y14" s="17">
+        <v>6</v>
+      </c>
       <c r="Z14" s="18"/>
       <c r="AA14" s="16"/>
       <c r="AB14" s="17"/>
@@ -4632,7 +4646,7 @@
       <c r="AG14" s="54"/>
       <c r="AH14" s="43">
         <f>SUM(C14:AG14)</f>
-        <v>46</v>
+        <v>73</v>
       </c>
     </row>
     <row r="15" spans="1:34" ht="15" customHeight="1">
@@ -17183,26 +17197,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0e61e294-5db2-4ad2-9356-7488524978e7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9160ec49-0786-419e-aae3-9c9cb8f5a974" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C289070B8F9CFE47959C16D84F6C625E" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="fe8aa3d2fe1a9c7effcd8e73d8f32c18">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0e61e294-5db2-4ad2-9356-7488524978e7" xmlns:ns3="9160ec49-0786-419e-aae3-9c9cb8f5a974" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d0f39d0209994a88c6a94a692ea058f4" ns2:_="" ns3:_="">
     <xsd:import namespace="0e61e294-5db2-4ad2-9356-7488524978e7"/>
@@ -17437,10 +17431,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0e61e294-5db2-4ad2-9356-7488524978e7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9160ec49-0786-419e-aae3-9c9cb8f5a974" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D23919C5-C77D-4D6C-8993-5ED5B021C1A8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2824570A-9196-4B56-8A33-38A1E7BF27D2}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="0e61e294-5db2-4ad2-9356-7488524978e7"/>
+    <ds:schemaRef ds:uri="9160ec49-0786-419e-aae3-9c9cb8f5a974"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -17459,20 +17484,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2824570A-9196-4B56-8A33-38A1E7BF27D2}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D23919C5-C77D-4D6C-8993-5ED5B021C1A8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="0e61e294-5db2-4ad2-9356-7488524978e7"/>
-    <ds:schemaRef ds:uri="9160ec49-0786-419e-aae3-9c9cb8f5a974"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Add confidence calibration and October month-end evidence
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project/StellaDev WBSO 2026 - Hours registration -  (ENG).xlsx
+++ b/project/StellaDev WBSO 2026 - Hours registration -  (ENG).xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10927"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11027"/>
   <workbookPr checkCompatibility="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/filippomargiotta/Documents/Personal/AosRepo/project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{321B8E83-E169-C14C-A022-8036F34741DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8335C3F7-74F2-1147-AB92-3F6452FF4534}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="32200" windowHeight="19920" tabRatio="666" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2103,7 +2103,7 @@
       </c>
       <c r="L12" s="70">
         <f>October!AH14</f>
-        <v>73</v>
+        <v>103</v>
       </c>
       <c r="M12" s="70">
         <f>November!AG14</f>
@@ -2115,7 +2115,7 @@
       </c>
       <c r="O12" s="69">
         <f>SUM(C12:N12)</f>
-        <v>935</v>
+        <v>965</v>
       </c>
     </row>
     <row r="13" spans="1:34" ht="15" customHeight="1">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="L29" s="5">
         <f t="shared" si="1"/>
-        <v>73</v>
+        <v>103</v>
       </c>
       <c r="M29" s="5">
         <f t="shared" si="1"/>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="O29" s="6">
         <f t="shared" si="1"/>
-        <v>935</v>
+        <v>965</v>
       </c>
     </row>
     <row r="31" spans="2:15" ht="15" customHeight="1">
@@ -4636,17 +4636,31 @@
       <c r="Y14" s="17">
         <v>6</v>
       </c>
-      <c r="Z14" s="18"/>
-      <c r="AA14" s="16"/>
-      <c r="AB14" s="17"/>
-      <c r="AC14" s="17"/>
-      <c r="AD14" s="17"/>
-      <c r="AE14" s="17"/>
-      <c r="AF14" s="17"/>
+      <c r="Z14" s="18">
+        <v>4</v>
+      </c>
+      <c r="AA14" s="16">
+        <v>4</v>
+      </c>
+      <c r="AB14" s="17">
+        <v>4</v>
+      </c>
+      <c r="AC14" s="17">
+        <v>6</v>
+      </c>
+      <c r="AD14" s="17">
+        <v>2</v>
+      </c>
+      <c r="AE14" s="17">
+        <v>4</v>
+      </c>
+      <c r="AF14" s="17">
+        <v>6</v>
+      </c>
       <c r="AG14" s="54"/>
       <c r="AH14" s="43">
         <f>SUM(C14:AG14)</f>
-        <v>73</v>
+        <v>103</v>
       </c>
     </row>
     <row r="15" spans="1:34" ht="15" customHeight="1">
@@ -17197,6 +17211,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0e61e294-5db2-4ad2-9356-7488524978e7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9160ec49-0786-419e-aae3-9c9cb8f5a974" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C289070B8F9CFE47959C16D84F6C625E" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="fe8aa3d2fe1a9c7effcd8e73d8f32c18">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0e61e294-5db2-4ad2-9356-7488524978e7" xmlns:ns3="9160ec49-0786-419e-aae3-9c9cb8f5a974" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d0f39d0209994a88c6a94a692ea058f4" ns2:_="" ns3:_="">
     <xsd:import namespace="0e61e294-5db2-4ad2-9356-7488524978e7"/>
@@ -17431,27 +17465,28 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0e61e294-5db2-4ad2-9356-7488524978e7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9160ec49-0786-419e-aae3-9c9cb8f5a974" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D23919C5-C77D-4D6C-8993-5ED5B021C1A8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1149BA22-2185-4279-8D4D-20B81C2A7999}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="a022c38d-a398-45a6-8336-4b22e89f761d"/>
+    <ds:schemaRef ds:uri="52db9a4d-0878-46fa-948e-68042efe192b"/>
+    <ds:schemaRef ds:uri="0e61e294-5db2-4ad2-9356-7488524978e7"/>
+    <ds:schemaRef ds:uri="9160ec49-0786-419e-aae3-9c9cb8f5a974"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2824570A-9196-4B56-8A33-38A1E7BF27D2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -17470,27 +17505,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1149BA22-2185-4279-8D4D-20B81C2A7999}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="a022c38d-a398-45a6-8336-4b22e89f761d"/>
-    <ds:schemaRef ds:uri="52db9a4d-0878-46fa-948e-68042efe192b"/>
-    <ds:schemaRef ds:uri="0e61e294-5db2-4ad2-9356-7488524978e7"/>
-    <ds:schemaRef ds:uri="9160ec49-0786-419e-aae3-9c9cb8f5a974"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D23919C5-C77D-4D6C-8993-5ED5B021C1A8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{0eea11ca-d417-4147-80ed-01a58412c458}" enabled="1" method="Standard" siteId="{bc9dc15c-61bc-4f03-b60b-e5b6d8922839}" contentBits="2" removed="0"/>

</xml_diff>